<commit_message>
Adding a few new jobs
</commit_message>
<xml_diff>
--- a/job-openings-scripts/muoniverse-job-openings.xlsx
+++ b/job-openings-scripts/muoniverse-job-openings.xlsx
@@ -137,7 +137,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="108">
   <si>
     <t>Role</t>
   </si>
@@ -416,6 +416,30 @@
   </si>
   <si>
     <t xml:space="preserve">Design of a secure data sharing portal for muon data</t>
+  </si>
+  <si>
+    <t>F5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paolo Crivelli </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Muonium spectroscopy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">potential internal candidate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peter Stoffer (PSI and UZH)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Advancing the theoretical framework for rare muon observables</t>
+  </si>
+  <si>
+    <t>T5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cryogenic detector to accurately track positrons from muon decays</t>
   </si>
   <si>
     <t xml:space="preserve">For any job offering, please add a row filling *all* columns</t>
@@ -504,7 +528,7 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1"/>
     <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
@@ -521,7 +545,6 @@
     </xf>
     <xf fontId="4" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
     <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="1" applyFont="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" quotePrefix="1"/>
     <xf fontId="2" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -545,8 +568,8 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="Pizzi, Giovanni" id="{754E0216-212F-1693-6280-CED5E2EB28B4}" userId="S::giovanni.pizzi@psi.ch::fcd49011-dac4-4c01-9bc6-eefdd0021243" providerId="AD"/>
-  <person displayName="Pizzi, Giovanni" id="{C049B3F4-A35B-7D00-0A87-C89CB440E4D8}" userId="S::giovanni.pizzi@psi.ch::fcd49011-dac4-4c01-9bc6-eefdd0021243" providerId="Teamlab"/>
+  <person displayName="Pizzi, Giovanni" id="{9C172AE7-2292-4967-A597-2F0F193C24EF}" userId="S::giovanni.pizzi@psi.ch::fcd49011-dac4-4c01-9bc6-eefdd0021243" providerId="AD"/>
+  <person displayName="Pizzi, Giovanni" id="{678EEF45-6297-14CE-DC81-31D46257F290}" userId="S::giovanni.pizzi@psi.ch::fcd49011-dac4-4c01-9bc6-eefdd0021243" providerId="Teamlab"/>
 </personList>
 </file>
 
@@ -1062,23 +1085,23 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="A1" dT="2026-02-02T10:18:20.32Z" personId="{754E0216-212F-1693-6280-CED5E2EB28B4}" id="{D3909E3A-CF3A-6144-B66D-EC5AECD54804}" done="0">
+  <threadedComment ref="A1" dT="2026-02-02T10:18:20.32Z" personId="{9C172AE7-2292-4967-A597-2F0F193C24EF}" id="{D3909E3A-CF3A-6144-B66D-EC5AECD54804}" done="0">
     <text xml:space="preserve">Please use standardized phrasing (copy from lines above, if needed)
 </text>
   </threadedComment>
-  <threadedComment ref="B1" dT="2026-02-02T10:18:52.37Z" personId="{754E0216-212F-1693-6280-CED5E2EB28B4}" id="{3A2C8F42-915E-4B42-8C35-1087C2FD6E67}" done="0">
+  <threadedComment ref="B1" dT="2026-02-02T10:18:52.37Z" personId="{9C172AE7-2292-4967-A597-2F0F193C24EF}" id="{3A2C8F42-915E-4B42-8C35-1087C2FD6E67}" done="0">
     <text xml:space="preserve">Please use standardized name (copy name from rows above, if one already exists)
 </text>
   </threadedComment>
-  <threadedComment ref="E1" dT="2026-02-02T10:19:08.34Z" personId="{C049B3F4-A35B-7D00-0A87-C89CB440E4D8}" id="{0DD1F034-F3C2-6143-B5EE-4D8ACB9B94D3}" done="0">
+  <threadedComment ref="E1" dT="2026-02-02T10:19:08.34Z" personId="{678EEF45-6297-14CE-DC81-31D46257F290}" id="{0DD1F034-F3C2-6143-B5EE-4D8ACB9B94D3}" done="0">
     <text xml:space="preserve">Short 1-line job description
 </text>
   </threadedComment>
-  <threadedComment ref="F1" dT="2026-02-02T10:19:37.74Z" personId="{C049B3F4-A35B-7D00-0A87-C89CB440E4D8}" id="{7B781CE5-788D-EE45-89AA-868478A6290E}" done="0">
+  <threadedComment ref="F1" dT="2026-02-02T10:19:37.74Z" personId="{678EEF45-6297-14CE-DC81-31D46257F290}" id="{7B781CE5-788D-EE45-89AA-868478A6290E}" done="0">
     <text xml:space="preserve">Direct link to page with full application (and link to apply). If not present, the button will not be shown
 </text>
   </threadedComment>
-  <threadedComment ref="G1" dT="2026-02-05T22:35:50.45Z" personId="{C049B3F4-A35B-7D00-0A87-C89CB440E4D8}" id="{803435A0-8165-0344-9437-CCA1C17B6D10}" done="0">
+  <threadedComment ref="G1" dT="2026-02-05T22:35:50.45Z" personId="{678EEF45-6297-14CE-DC81-31D46257F290}" id="{803435A0-8165-0344-9437-CCA1C17B6D10}" done="0">
     <text xml:space="preserve">When the date is in the past, the job ad will not be shown.
 Not required if the link is not yet present
 </text>
@@ -1100,7 +1123,7 @@
     <col bestFit="1" customWidth="1" min="8" max="8" width="44.83203125"/>
   </cols>
   <sheetData>
-    <row r="1" ht="13.85">
+    <row r="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1126,7 +1149,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" ht="13.85">
+    <row r="2">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -1143,7 +1166,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" ht="13.85">
+    <row r="3" ht="15">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1166,7 +1189,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" ht="13.85">
+    <row r="4" ht="15">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1183,7 +1206,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" ht="13.85">
+    <row r="5" ht="15">
       <c r="A5" s="4" t="s">
         <v>22</v>
       </c>
@@ -1226,7 +1249,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" ht="13.85">
+    <row r="7" ht="15">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1243,7 +1266,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8" ht="13.85">
+    <row r="8" ht="15">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -1260,7 +1283,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" ht="13.85">
+    <row r="9" ht="15">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -1280,7 +1303,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="10" ht="13.85">
+    <row r="10" ht="15">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -1297,7 +1320,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="11" ht="13.85">
+    <row r="11" ht="15">
       <c r="A11" t="s">
         <v>26</v>
       </c>
@@ -1314,7 +1337,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="12" ht="13.85">
+    <row r="12" ht="15">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -1330,9 +1353,8 @@
       <c r="E12" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="G12" s="1"/>
-    </row>
-    <row r="13" ht="13.85">
+    </row>
+    <row r="13" ht="15">
       <c r="A13" t="s">
         <v>8</v>
       </c>
@@ -1355,7 +1377,7 @@
         <v>46127</v>
       </c>
     </row>
-    <row r="14" ht="13.85">
+    <row r="14" ht="15">
       <c r="A14" t="s">
         <v>8</v>
       </c>
@@ -1372,7 +1394,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="15" ht="13.85">
+    <row r="15" ht="15">
       <c r="A15" t="s">
         <v>26</v>
       </c>
@@ -1395,7 +1417,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="16" ht="13.85">
+    <row r="16" ht="15">
       <c r="A16" t="s">
         <v>8</v>
       </c>
@@ -1412,7 +1434,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="17" ht="13.85">
+    <row r="17" ht="15">
       <c r="A17" t="s">
         <v>8</v>
       </c>
@@ -1429,7 +1451,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="18" ht="13.85">
+    <row r="18" ht="15">
       <c r="A18" t="s">
         <v>8</v>
       </c>
@@ -1446,7 +1468,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="19" ht="13.85">
+    <row r="19" ht="15">
       <c r="A19" s="7" t="s">
         <v>8</v>
       </c>
@@ -1463,7 +1485,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="20" ht="13.85">
+    <row r="20" ht="15">
       <c r="A20" s="7" t="s">
         <v>26</v>
       </c>
@@ -1480,7 +1502,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="21" ht="13.85">
+    <row r="21" ht="15">
       <c r="A21" t="s">
         <v>26</v>
       </c>
@@ -1497,7 +1519,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="22" ht="13.85">
+    <row r="22" ht="15">
       <c r="A22" t="s">
         <v>8</v>
       </c>
@@ -1514,14 +1536,14 @@
         <v>81</v>
       </c>
     </row>
-    <row r="23" ht="13.85">
+    <row r="23" ht="15">
       <c r="A23" t="s">
         <v>26</v>
       </c>
       <c r="B23" t="s">
         <v>82</v>
       </c>
-      <c r="C23" s="10" t="s">
+      <c r="C23" t="s">
         <v>83</v>
       </c>
       <c r="D23" t="s">
@@ -1531,7 +1553,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="24" ht="13.85">
+    <row r="24" ht="15">
       <c r="A24" t="s">
         <v>26</v>
       </c>
@@ -1551,14 +1573,14 @@
         <v>88</v>
       </c>
     </row>
-    <row r="25" ht="13.85">
+    <row r="25" ht="15">
       <c r="A25" t="s">
         <v>89</v>
       </c>
       <c r="B25" t="s">
         <v>9</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="C25" s="4" t="s">
         <v>90</v>
       </c>
       <c r="D25" t="s">
@@ -1567,10 +1589,63 @@
       <c r="E25" t="s">
         <v>92</v>
       </c>
-      <c r="F25" s="11"/>
+      <c r="F25" s="10"/>
       <c r="G25" s="1"/>
     </row>
-    <row r="26" ht="13.85"/>
+    <row r="26" ht="15">
+      <c r="A26" t="s">
+        <v>8</v>
+      </c>
+      <c r="B26" t="s">
+        <v>55</v>
+      </c>
+      <c r="C26" t="s">
+        <v>93</v>
+      </c>
+      <c r="D26" t="s">
+        <v>94</v>
+      </c>
+      <c r="E26" t="s">
+        <v>95</v>
+      </c>
+      <c r="H26" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="27" ht="15">
+      <c r="A27" t="s">
+        <v>8</v>
+      </c>
+      <c r="B27" t="s">
+        <v>9</v>
+      </c>
+      <c r="C27" t="s">
+        <v>41</v>
+      </c>
+      <c r="D27" t="s">
+        <v>97</v>
+      </c>
+      <c r="E27" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="28" ht="15">
+      <c r="A28" t="s">
+        <v>26</v>
+      </c>
+      <c r="B28" t="s">
+        <v>9</v>
+      </c>
+      <c r="C28" t="s">
+        <v>99</v>
+      </c>
+      <c r="D28" t="s">
+        <v>42</v>
+      </c>
+      <c r="E28" t="s">
+        <v>100</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="F6" tooltip="https://www.unifr.ch/phys/en/department/jobs/"/>
@@ -1594,37 +1669,37 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="s">
-        <v>95</v>
+      <c r="A4" s="11" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="s">
-        <v>96</v>
+      <c r="A5" s="11" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="s">
-        <v>97</v>
+      <c r="A6" s="11" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="s">
-        <v>98</v>
+      <c r="A7" s="11" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="s">
-        <v>99</v>
+      <c r="A9" s="12" t="s">
+        <v>107</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
New job, and a bit more automation
</commit_message>
<xml_diff>
--- a/job-openings-scripts/muoniverse-job-openings.xlsx
+++ b/job-openings-scripts/muoniverse-job-openings.xlsx
@@ -137,7 +137,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="122">
   <si>
     <t>Role</t>
   </si>
@@ -187,6 +187,21 @@
     <t>https://www.psi.ch/de/hr/stellenangebote/74283-assistentin-50-100</t>
   </si>
   <si>
+    <t xml:space="preserve">Technical Scientific Staff Member</t>
+  </si>
+  <si>
+    <t xml:space="preserve">University of Zurich</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marc Janoschek (UZH), Fabian Natterer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Managing the Quantum Sensing Platform (QSP) for Muoniverse at the Department of Physics at University of Zurich</t>
+  </si>
+  <si>
+    <t>https://apply.mnf.uzh.ch/auth/2%3A1%3A0%3A0%3A0%3A_csrf%3A3c924364-f1dd-4211-a334-72e84c13cdd0/</t>
+  </si>
+  <si>
     <t xml:space="preserve">PhD Student</t>
   </si>
   <si>
@@ -199,9 +214,6 @@
     <t xml:space="preserve">Quantum-mechanical simulations of muons in materials</t>
   </si>
   <si>
-    <t xml:space="preserve">University of Zurich</t>
-  </si>
-  <si>
     <t>F1,T7</t>
   </si>
   <si>
@@ -370,10 +382,13 @@
     <t xml:space="preserve">University of Zürich</t>
   </si>
   <si>
-    <t xml:space="preserve">Fabian Naterrer</t>
+    <t xml:space="preserve">Fabian Natterer (UZH)</t>
   </si>
   <si>
     <t xml:space="preserve">Hunting for hints for time-reversal symmetry-breaking superconductivity in Josephosn Junction STM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">internal candidate, start 1. September 2026</t>
   </si>
   <si>
     <t>T1</t>
@@ -595,8 +610,8 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="Pizzi, Giovanni" id="{BF6B20CA-7F05-D35D-BB2F-A14D616340A2}" userId="S::giovanni.pizzi@psi.ch::fcd49011-dac4-4c01-9bc6-eefdd0021243" providerId="AD"/>
-  <person displayName="Pizzi, Giovanni" id="{99C125A3-A489-092C-708E-6C6675608153}" userId="S::giovanni.pizzi@psi.ch::fcd49011-dac4-4c01-9bc6-eefdd0021243" providerId="Teamlab"/>
+  <person displayName="Pizzi, Giovanni" id="{8F48D80C-62CA-3A15-B339-8D50D0466734}" userId="S::giovanni.pizzi@psi.ch::fcd49011-dac4-4c01-9bc6-eefdd0021243" providerId="AD"/>
+  <person displayName="Pizzi, Giovanni" id="{A030E1C5-7CEB-E74A-16EA-FFF64B3B7C13}" userId="S::giovanni.pizzi@psi.ch::fcd49011-dac4-4c01-9bc6-eefdd0021243" providerId="Teamlab"/>
 </personList>
 </file>
 
@@ -1112,23 +1127,23 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="A1" dT="2026-02-02T10:18:20.32Z" personId="{BF6B20CA-7F05-D35D-BB2F-A14D616340A2}" id="{D3909E3A-CF3A-6144-B66D-EC5AECD54804}" done="0">
+  <threadedComment ref="A1" dT="2026-02-02T10:18:20.32Z" personId="{8F48D80C-62CA-3A15-B339-8D50D0466734}" id="{D3909E3A-CF3A-6144-B66D-EC5AECD54804}" done="0">
     <text xml:space="preserve">Please use standardized phrasing (copy from lines above, if needed)
 </text>
   </threadedComment>
-  <threadedComment ref="B1" dT="2026-02-02T10:18:52.37Z" personId="{BF6B20CA-7F05-D35D-BB2F-A14D616340A2}" id="{3A2C8F42-915E-4B42-8C35-1087C2FD6E67}" done="0">
+  <threadedComment ref="B1" dT="2026-02-02T10:18:52.37Z" personId="{8F48D80C-62CA-3A15-B339-8D50D0466734}" id="{3A2C8F42-915E-4B42-8C35-1087C2FD6E67}" done="0">
     <text xml:space="preserve">Please use standardized name (copy name from rows above, if one already exists)
 </text>
   </threadedComment>
-  <threadedComment ref="E1" dT="2026-02-02T10:19:08.34Z" personId="{99C125A3-A489-092C-708E-6C6675608153}" id="{0DD1F034-F3C2-6143-B5EE-4D8ACB9B94D3}" done="0">
+  <threadedComment ref="E1" dT="2026-02-02T10:19:08.34Z" personId="{A030E1C5-7CEB-E74A-16EA-FFF64B3B7C13}" id="{0DD1F034-F3C2-6143-B5EE-4D8ACB9B94D3}" done="0">
     <text xml:space="preserve">Short 1-line job description
 </text>
   </threadedComment>
-  <threadedComment ref="F1" dT="2026-02-02T10:19:37.74Z" personId="{99C125A3-A489-092C-708E-6C6675608153}" id="{7B781CE5-788D-EE45-89AA-868478A6290E}" done="0">
+  <threadedComment ref="F1" dT="2026-02-02T10:19:37.74Z" personId="{A030E1C5-7CEB-E74A-16EA-FFF64B3B7C13}" id="{7B781CE5-788D-EE45-89AA-868478A6290E}" done="0">
     <text xml:space="preserve">Direct link to page with full application (and link to apply). If not present, the button will not be shown
 </text>
   </threadedComment>
-  <threadedComment ref="G1" dT="2026-02-05T22:35:50.45Z" personId="{99C125A3-A489-092C-708E-6C6675608153}" id="{803435A0-8165-0344-9437-CCA1C17B6D10}" done="0">
+  <threadedComment ref="G1" dT="2026-02-05T22:35:50.45Z" personId="{A030E1C5-7CEB-E74A-16EA-FFF64B3B7C13}" id="{803435A0-8165-0344-9437-CCA1C17B6D10}" done="0">
     <text xml:space="preserve">When the date is in the past, the job ad will not be shown.
 Not required if the link is not yet present
 </text>
@@ -1140,7 +1155,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13.880000000000001"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="23.83203125"/>
+    <col customWidth="1" min="1" max="1" width="77.77734375"/>
     <col bestFit="1" customWidth="1" min="2" max="2" width="28.50390625"/>
     <col customWidth="1" min="3" max="3" width="29.21484375"/>
     <col customWidth="1" min="4" max="4" width="52.21484375"/>
@@ -1150,7 +1165,7 @@
     <col bestFit="1" customWidth="1" min="8" max="8" width="44.83203125"/>
   </cols>
   <sheetData>
-    <row r="1" ht="13.85">
+    <row r="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1176,7 +1191,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" ht="13.85">
+    <row r="2">
       <c r="A2" s="4" t="s">
         <v>8</v>
       </c>
@@ -1197,7 +1212,7 @@
       </c>
       <c r="H2" s="4"/>
     </row>
-    <row r="3" s="0" customFormat="1" ht="13.85">
+    <row r="3" s="0" customFormat="1">
       <c r="A3" s="4" t="s">
         <v>13</v>
       </c>
@@ -1217,166 +1232,164 @@
         <v>46142</v>
       </c>
     </row>
-    <row r="4" ht="13.85">
-      <c r="A4" t="s">
+    <row r="4" s="0" customFormat="1">
+      <c r="A4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G4" s="1"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" ht="15">
+      <c r="A6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" t="s">
         <v>17</v>
       </c>
-      <c r="D4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" ht="13.85">
-      <c r="A5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" s="4" t="s">
+      <c r="C6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G6" s="1">
+        <v>46029</v>
+      </c>
+      <c r="H6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" ht="15">
+      <c r="A7" t="s">
         <v>21</v>
       </c>
-      <c r="D5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E5" t="s">
-        <v>23</v>
-      </c>
-      <c r="G5" s="1">
+      <c r="B7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" ht="15">
+      <c r="A8" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="E8" t="s">
+        <v>32</v>
+      </c>
+      <c r="G8" s="1">
         <v>46029</v>
       </c>
-      <c r="H5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6" ht="13.85">
-      <c r="A6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D6" t="s">
-        <v>27</v>
-      </c>
-      <c r="E6" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="7" ht="13.85">
-      <c r="A7" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="E7" t="s">
-        <v>28</v>
-      </c>
-      <c r="G7" s="1">
-        <v>46029</v>
-      </c>
-      <c r="H7" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="8" ht="16.5" customHeight="1">
-      <c r="A8" t="s">
-        <v>33</v>
-      </c>
-      <c r="B8" t="s">
-        <v>34</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D8" t="s">
+      <c r="H8" t="s">
         <v>36</v>
       </c>
-      <c r="E8" s="8" t="s">
+    </row>
+    <row r="9" ht="16.5" customHeight="1">
+      <c r="A9" t="s">
         <v>37</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="B9" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="9" ht="13.85">
-      <c r="A9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9" t="s">
+      <c r="C9" s="4" t="s">
         <v>39</v>
       </c>
       <c r="D9" t="s">
         <v>40</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="8" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="10" ht="13.85">
+      <c r="F9" s="6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="10" ht="15">
       <c r="A10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="5" t="s">
-        <v>42</v>
+      <c r="C10" t="s">
+        <v>43</v>
       </c>
       <c r="D10" t="s">
-        <v>40</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="11" ht="13.85">
+        <v>44</v>
+      </c>
+      <c r="E10" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11" ht="15">
       <c r="A11" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" t="s">
-        <v>20</v>
-      </c>
-      <c r="C11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D11" t="s">
         <v>44</v>
       </c>
-      <c r="D11" t="s">
-        <v>45</v>
-      </c>
-      <c r="E11" t="s">
-        <v>46</v>
-      </c>
-      <c r="F11" s="7" t="s">
+      <c r="E11" s="5" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="12" ht="13.85">
+    <row r="12" ht="15">
       <c r="A12" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B12" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="C12" t="s">
         <v>48</v>
@@ -1384,50 +1397,53 @@
       <c r="D12" t="s">
         <v>49</v>
       </c>
-      <c r="E12" s="8" t="s">
+      <c r="E12" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="13" ht="13.85">
+      <c r="F12" s="7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="13" ht="15">
       <c r="A13" t="s">
-        <v>33</v>
-      </c>
-      <c r="B13" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" t="s">
         <v>9</v>
       </c>
       <c r="C13" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D13" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="14" ht="13.85">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="14" ht="15">
       <c r="A14" t="s">
-        <v>16</v>
-      </c>
-      <c r="B14" t="s">
+        <v>37</v>
+      </c>
+      <c r="B14" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D14" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="15" ht="13.85">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="15" ht="15">
       <c r="A15" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B15" t="s">
-        <v>57</v>
+        <v>9</v>
       </c>
       <c r="C15" t="s">
         <v>58</v>
@@ -1435,36 +1451,36 @@
       <c r="D15" t="s">
         <v>59</v>
       </c>
-      <c r="E15" s="9" t="s">
+      <c r="E15" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="F15" s="7" t="s">
+    </row>
+    <row r="16" ht="15">
+      <c r="A16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" t="s">
         <v>61</v>
       </c>
-      <c r="G15" s="1">
+      <c r="C16" t="s">
+        <v>62</v>
+      </c>
+      <c r="D16" t="s">
+        <v>63</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="G16" s="1">
         <v>46127</v>
       </c>
     </row>
-    <row r="16" ht="13.85">
-      <c r="A16" t="s">
-        <v>16</v>
-      </c>
-      <c r="B16" t="s">
-        <v>62</v>
-      </c>
-      <c r="C16" t="s">
-        <v>63</v>
-      </c>
-      <c r="D16" t="s">
-        <v>64</v>
-      </c>
-      <c r="E16" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="17" ht="13.85">
+    <row r="17" ht="15">
       <c r="A17" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B17" t="s">
         <v>66</v>
@@ -1478,19 +1494,13 @@
       <c r="E17" t="s">
         <v>69</v>
       </c>
-      <c r="G17" s="1">
-        <v>46143</v>
-      </c>
-      <c r="H17" t="s">
+    </row>
+    <row r="18" ht="15">
+      <c r="A18" t="s">
+        <v>37</v>
+      </c>
+      <c r="B18" t="s">
         <v>70</v>
-      </c>
-    </row>
-    <row r="18" ht="13.85">
-      <c r="A18" t="s">
-        <v>16</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>9</v>
       </c>
       <c r="C18" t="s">
         <v>71</v>
@@ -1498,252 +1508,283 @@
       <c r="D18" t="s">
         <v>72</v>
       </c>
-      <c r="E18" s="5" t="s">
+      <c r="E18" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="19" ht="13.85">
+      <c r="G18" s="1">
+        <v>46143</v>
+      </c>
+      <c r="H18" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="19" ht="15">
       <c r="A19" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>66</v>
+        <v>9</v>
       </c>
       <c r="C19" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D19" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E19" s="5" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="20" ht="15">
+      <c r="A20" t="s">
+        <v>21</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="C20" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="20" ht="13.85">
-      <c r="A20" t="s">
-        <v>16</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C20" t="s">
-        <v>71</v>
-      </c>
       <c r="D20" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="21" ht="13.85">
-      <c r="A21" s="5" t="s">
-        <v>16</v>
+        <v>79</v>
+      </c>
+      <c r="G20" s="1"/>
+    </row>
+    <row r="21" ht="15">
+      <c r="A21" t="s">
+        <v>21</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>9</v>
+        <v>80</v>
       </c>
       <c r="C21" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="D21" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="22" ht="13.85">
+        <v>82</v>
+      </c>
+      <c r="G21" s="1">
+        <v>46266</v>
+      </c>
+      <c r="H21" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="22" ht="15">
       <c r="A22" s="5" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C22" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="D22" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="23" ht="13.85">
-      <c r="A23" t="s">
-        <v>33</v>
+        <v>86</v>
+      </c>
+    </row>
+    <row r="23" ht="15">
+      <c r="A23" s="5" t="s">
+        <v>37</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C23" t="s">
-        <v>82</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="E23" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="24" ht="13.85">
+      <c r="D23" t="s">
+        <v>85</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="24" ht="15">
       <c r="A24" t="s">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>85</v>
+        <v>9</v>
       </c>
       <c r="C24" t="s">
-        <v>86</v>
-      </c>
-      <c r="D24" t="s">
         <v>87</v>
       </c>
-      <c r="E24" s="4" t="s">
+      <c r="D24" s="5" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="25" ht="13.85">
+      <c r="E24" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="25" ht="15">
       <c r="A25" t="s">
-        <v>33</v>
-      </c>
-      <c r="B25" t="s">
-        <v>89</v>
+        <v>21</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>90</v>
       </c>
       <c r="C25" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D25" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="26" ht="13.85">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="26" ht="15">
       <c r="A26" t="s">
-        <v>33</v>
-      </c>
-      <c r="B26" s="5" t="s">
-        <v>9</v>
+        <v>37</v>
+      </c>
+      <c r="B26" t="s">
+        <v>94</v>
       </c>
       <c r="C26" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D26" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
       <c r="E26" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="H26" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="27" ht="13.85">
+    </row>
+    <row r="27" ht="15">
       <c r="A27" t="s">
-        <v>95</v>
-      </c>
-      <c r="B27" t="s">
+        <v>37</v>
+      </c>
+      <c r="B27" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C27" s="4" t="s">
-        <v>96</v>
+      <c r="C27" t="s">
+        <v>97</v>
       </c>
       <c r="D27" t="s">
-        <v>97</v>
-      </c>
-      <c r="E27" t="s">
+        <v>10</v>
+      </c>
+      <c r="E27" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="F27" s="10"/>
-      <c r="G27" s="1"/>
-    </row>
-    <row r="28" ht="13.85">
+      <c r="H27" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="28" ht="15">
       <c r="A28" t="s">
-        <v>16</v>
+        <v>100</v>
       </c>
       <c r="B28" t="s">
-        <v>62</v>
-      </c>
-      <c r="C28" t="s">
-        <v>99</v>
+        <v>9</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>101</v>
       </c>
       <c r="D28" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E28" t="s">
-        <v>101</v>
-      </c>
-      <c r="H28" s="5" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="29" ht="13.85">
+        <v>103</v>
+      </c>
+      <c r="F28" s="10"/>
+      <c r="G28" s="1"/>
+    </row>
+    <row r="29" ht="15">
       <c r="A29" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B29" t="s">
-        <v>9</v>
+        <v>66</v>
       </c>
       <c r="C29" t="s">
-        <v>48</v>
+        <v>104</v>
       </c>
       <c r="D29" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E29" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="30" ht="13.85">
+        <v>106</v>
+      </c>
+      <c r="H29" s="5" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="30" ht="15">
       <c r="A30" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B30" t="s">
         <v>9</v>
       </c>
       <c r="C30" t="s">
-        <v>105</v>
+        <v>52</v>
       </c>
       <c r="D30" t="s">
-        <v>49</v>
+        <v>108</v>
       </c>
       <c r="E30" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="31" ht="13.85">
-      <c r="A31" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="B31" s="5" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="31" ht="15">
+      <c r="A31" t="s">
+        <v>37</v>
+      </c>
+      <c r="B31" t="s">
         <v>9</v>
       </c>
       <c r="C31" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="D31" t="s">
-        <v>108</v>
+        <v>53</v>
       </c>
       <c r="E31" t="s">
-        <v>109</v>
+        <v>111</v>
+      </c>
+    </row>
+    <row r="32" ht="15">
+      <c r="A32" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C32" t="s">
+        <v>112</v>
+      </c>
+      <c r="D32" t="s">
+        <v>113</v>
+      </c>
+      <c r="E32" t="s">
+        <v>114</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="F2" tooltip=""/>
     <hyperlink r:id="rId2" ref="F3"/>
-    <hyperlink r:id="rId3" ref="F8" tooltip="https://www.unifr.ch/phys/en/department/jobs/"/>
-    <hyperlink r:id="rId4" ref="F11"/>
-    <hyperlink r:id="rId5" ref="F15"/>
+    <hyperlink r:id="rId3" ref="F4"/>
+    <hyperlink r:id="rId4" ref="F9" tooltip="https://www.unifr.ch/phys/en/department/jobs/"/>
+    <hyperlink r:id="rId5" ref="F12"/>
+    <hyperlink r:id="rId6" ref="F16"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="0" verticalDpi="0" copies="1"/>
   <headerFooter/>
-  <legacyDrawing r:id="rId8"/>
+  <legacyDrawing r:id="rId9"/>
 </worksheet>
 </file>
 
@@ -1756,37 +1797,37 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="11" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adding 2 new openings
</commit_message>
<xml_diff>
--- a/job-openings-scripts/muoniverse-job-openings.xlsx
+++ b/job-openings-scripts/muoniverse-job-openings.xlsx
@@ -137,7 +137,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="131">
   <si>
     <t>Role</t>
   </si>
@@ -316,6 +316,9 @@
     <t xml:space="preserve">Development of μSR pressure cells for quantum materials research</t>
   </si>
   <si>
+    <t>https://www.psi.ch/en/hr/job-opportunities/74376-postdoctoral-fellow-in-experimental-physics</t>
+  </si>
+  <si>
     <t>T6,F1</t>
   </si>
   <si>
@@ -323,6 +326,9 @@
   </si>
   <si>
     <t xml:space="preserve">Uniaxial and hydrostatic pressure studies on quantum materials </t>
+  </si>
+  <si>
+    <t>https://www.psi.ch/en/hr/job-opportunities/74375-phd-student-in-experimental-physics</t>
   </si>
   <si>
     <t>EPFL</t>
@@ -631,8 +637,8 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="Pizzi, Giovanni" id="{B9A76892-18E3-158B-1737-AD3BC9EB0620}" userId="S::giovanni.pizzi@psi.ch::fcd49011-dac4-4c01-9bc6-eefdd0021243" providerId="AD"/>
-  <person displayName="Pizzi, Giovanni" id="{AD773D16-1A25-7EB2-2CA9-67082C65F66B}" userId="S::giovanni.pizzi@psi.ch::fcd49011-dac4-4c01-9bc6-eefdd0021243" providerId="Teamlab"/>
+  <person displayName="Pizzi, Giovanni" id="{6922F27C-BE0C-7399-14F1-F78F015972B1}" userId="S::giovanni.pizzi@psi.ch::fcd49011-dac4-4c01-9bc6-eefdd0021243" providerId="AD"/>
+  <person displayName="Pizzi, Giovanni" id="{DC79B204-8000-E0C1-D3CC-5CF54A964D2F}" userId="S::giovanni.pizzi@psi.ch::fcd49011-dac4-4c01-9bc6-eefdd0021243" providerId="Teamlab"/>
 </personList>
 </file>
 
@@ -1148,23 +1154,23 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="A1" dT="2026-02-02T10:18:20.32Z" personId="{B9A76892-18E3-158B-1737-AD3BC9EB0620}" id="{D3909E3A-CF3A-6144-B66D-EC5AECD54804}" done="0">
+  <threadedComment ref="A1" dT="2026-02-02T10:18:20.32Z" personId="{6922F27C-BE0C-7399-14F1-F78F015972B1}" id="{D3909E3A-CF3A-6144-B66D-EC5AECD54804}" done="0">
     <text xml:space="preserve">Please use standardized phrasing (copy from lines above, if needed)
 </text>
   </threadedComment>
-  <threadedComment ref="B1" dT="2026-02-02T10:18:52.37Z" personId="{B9A76892-18E3-158B-1737-AD3BC9EB0620}" id="{3A2C8F42-915E-4B42-8C35-1087C2FD6E67}" done="0">
+  <threadedComment ref="B1" dT="2026-02-02T10:18:52.37Z" personId="{6922F27C-BE0C-7399-14F1-F78F015972B1}" id="{3A2C8F42-915E-4B42-8C35-1087C2FD6E67}" done="0">
     <text xml:space="preserve">Please use standardized name (copy name from rows above, if one already exists)
 </text>
   </threadedComment>
-  <threadedComment ref="E1" dT="2026-02-02T10:19:08.34Z" personId="{AD773D16-1A25-7EB2-2CA9-67082C65F66B}" id="{0DD1F034-F3C2-6143-B5EE-4D8ACB9B94D3}" done="0">
+  <threadedComment ref="E1" dT="2026-02-02T10:19:08.34Z" personId="{DC79B204-8000-E0C1-D3CC-5CF54A964D2F}" id="{0DD1F034-F3C2-6143-B5EE-4D8ACB9B94D3}" done="0">
     <text xml:space="preserve">Short 1-line job description
 </text>
   </threadedComment>
-  <threadedComment ref="F1" dT="2026-02-02T10:19:37.74Z" personId="{AD773D16-1A25-7EB2-2CA9-67082C65F66B}" id="{7B781CE5-788D-EE45-89AA-868478A6290E}" done="0">
+  <threadedComment ref="F1" dT="2026-02-02T10:19:37.74Z" personId="{DC79B204-8000-E0C1-D3CC-5CF54A964D2F}" id="{7B781CE5-788D-EE45-89AA-868478A6290E}" done="0">
     <text xml:space="preserve">Direct link to page with full application (and link to apply). If not present, the button will not be shown
 </text>
   </threadedComment>
-  <threadedComment ref="G1" dT="2026-02-05T22:35:50.45Z" personId="{AD773D16-1A25-7EB2-2CA9-67082C65F66B}" id="{803435A0-8165-0344-9437-CCA1C17B6D10}" done="0">
+  <threadedComment ref="G1" dT="2026-02-05T22:35:50.45Z" personId="{DC79B204-8000-E0C1-D3CC-5CF54A964D2F}" id="{803435A0-8165-0344-9437-CCA1C17B6D10}" done="0">
     <text xml:space="preserve">When the date is in the past, the job ad will not be shown.
 Not required if the link is not yet present
 </text>
@@ -1463,6 +1469,9 @@
       <c r="E14" s="8" t="s">
         <v>58</v>
       </c>
+      <c r="F14" s="7" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="15" ht="15">
       <c r="A15" t="s">
@@ -1472,13 +1481,16 @@
         <v>9</v>
       </c>
       <c r="C15" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D15" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>61</v>
+        <v>62</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="16" ht="15">
@@ -1486,19 +1498,19 @@
         <v>22</v>
       </c>
       <c r="B16" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C16" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D16" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="G16" s="1">
         <v>46127</v>
@@ -1509,16 +1521,16 @@
         <v>22</v>
       </c>
       <c r="B17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C17" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D17" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E17" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="18" ht="15">
@@ -1526,22 +1538,22 @@
         <v>38</v>
       </c>
       <c r="B18" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C18" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D18" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E18" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G18" s="1">
         <v>46143</v>
       </c>
       <c r="H18" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="19" ht="15">
@@ -1552,13 +1564,13 @@
         <v>9</v>
       </c>
       <c r="C19" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D19" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="20" ht="15">
@@ -1566,16 +1578,16 @@
         <v>22</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C20" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D20" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G20" s="1"/>
     </row>
@@ -1584,22 +1596,22 @@
         <v>22</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C21" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D21" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="G21" s="1">
         <v>46266</v>
       </c>
       <c r="H21" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="22" ht="15">
@@ -1610,13 +1622,13 @@
         <v>9</v>
       </c>
       <c r="C22" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D22" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="23" ht="15">
@@ -1627,13 +1639,13 @@
         <v>9</v>
       </c>
       <c r="C23" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D23" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="24" ht="15">
@@ -1644,13 +1656,13 @@
         <v>9</v>
       </c>
       <c r="C24" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E24" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="25" ht="15">
@@ -1658,16 +1670,16 @@
         <v>22</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C25" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D25" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="26" ht="15">
@@ -1675,19 +1687,19 @@
         <v>38</v>
       </c>
       <c r="B26" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C26" t="s">
+        <v>98</v>
+      </c>
+      <c r="D26" t="s">
+        <v>99</v>
+      </c>
+      <c r="E26" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="D26" t="s">
-        <v>97</v>
-      </c>
-      <c r="E26" s="4" t="s">
-        <v>94</v>
-      </c>
       <c r="F26" s="7" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G26" s="1">
         <v>46111</v>
@@ -1701,33 +1713,33 @@
         <v>9</v>
       </c>
       <c r="C27" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D27" t="s">
         <v>10</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="H27" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="28" ht="15">
       <c r="A28" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B28" t="s">
         <v>9</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D28" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E28" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F28" s="10"/>
       <c r="G28" s="1"/>
@@ -1737,19 +1749,19 @@
         <v>22</v>
       </c>
       <c r="B29" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C29" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D29" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E29" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="30" ht="15">
@@ -1763,10 +1775,10 @@
         <v>53</v>
       </c>
       <c r="D30" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E30" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="31" ht="15">
@@ -1777,13 +1789,13 @@
         <v>9</v>
       </c>
       <c r="C31" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D31" t="s">
         <v>54</v>
       </c>
       <c r="E31" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="32" ht="15">
@@ -1794,16 +1806,16 @@
         <v>9</v>
       </c>
       <c r="C32" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D32" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E32" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F32" s="7" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="33" ht="15">
@@ -1817,10 +1829,10 @@
         <v>40</v>
       </c>
       <c r="D33" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="E33" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="34" ht="15">
@@ -1834,10 +1846,10 @@
         <v>47</v>
       </c>
       <c r="D34" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E34" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="35" ht="15"/>
@@ -1848,15 +1860,17 @@
     <hyperlink r:id="rId3" ref="F4"/>
     <hyperlink r:id="rId4" ref="F9" tooltip="https://www.unifr.ch/phys/en/department/jobs/"/>
     <hyperlink r:id="rId5" ref="F12"/>
-    <hyperlink r:id="rId6" ref="F16"/>
-    <hyperlink r:id="rId7" ref="F26"/>
-    <hyperlink r:id="rId8" ref="F32"/>
+    <hyperlink r:id="rId6" ref="F14"/>
+    <hyperlink r:id="rId7" ref="F15"/>
+    <hyperlink r:id="rId8" ref="F16"/>
+    <hyperlink r:id="rId9" ref="F26"/>
+    <hyperlink r:id="rId10" ref="F32"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="0" verticalDpi="0" copies="1"/>
   <headerFooter/>
-  <legacyDrawing r:id="rId11"/>
+  <legacyDrawing r:id="rId13"/>
 </worksheet>
 </file>
 
@@ -1869,37 +1883,37 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="11" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: remove Low-energy muon spin rotation studies postdoc position
</commit_message>
<xml_diff>
--- a/job-openings-scripts/muoniverse-job-openings.xlsx
+++ b/job-openings-scripts/muoniverse-job-openings.xlsx
@@ -1,18 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/clange/muoniverse/website/job-openings-scripts/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55015865-5A55-2146-B4DD-757D562248FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
+    <workbookView xWindow="360" yWindow="780" windowWidth="32580" windowHeight="18500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Openings" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="Instructions" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="Openings" sheetId="1" r:id="rId1"/>
+    <sheet name="Instructions" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -26,110 +30,50 @@
     <author>tc={803435A0-8165-0344-9437-CCA1C17B6D10}</author>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0" xr:uid="{D3909E3A-CF3A-6144-B66D-EC5AECD54804}">
+    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{D3909E3A-CF3A-6144-B66D-EC5AECD54804}">
       <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Pizzi, Giovanni:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">
-Please use standardized phrasing (copy from lines above, if needed)
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Please use standardized phrasing (copy from lines above, if needed)
 </t>
-        </r>
       </text>
     </comment>
-    <comment ref="B1" authorId="1" xr:uid="{3A2C8F42-915E-4B42-8C35-1087C2FD6E67}">
+    <comment ref="B1" authorId="1" shapeId="0" xr:uid="{3A2C8F42-915E-4B42-8C35-1087C2FD6E67}">
       <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Pizzi, Giovanni:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">
-Please use standardized name (copy name from rows above, if one already exists)
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Please use standardized name (copy name from rows above, if one already exists)
 </t>
-        </r>
       </text>
     </comment>
-    <comment ref="E1" authorId="2" xr:uid="{0DD1F034-F3C2-6143-B5EE-4D8ACB9B94D3}">
+    <comment ref="E1" authorId="2" shapeId="0" xr:uid="{0DD1F034-F3C2-6143-B5EE-4D8ACB9B94D3}">
       <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Pizzi, Giovanni:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">
-Short 1-line job description
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Short 1-line job description
 </t>
-        </r>
       </text>
     </comment>
-    <comment ref="F1" authorId="3" xr:uid="{7B781CE5-788D-EE45-89AA-868478A6290E}">
+    <comment ref="F1" authorId="3" shapeId="0" xr:uid="{7B781CE5-788D-EE45-89AA-868478A6290E}">
       <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Pizzi, Giovanni:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">
-Direct link to page with full application (and link to apply). If not present, the button will not be shown
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Direct link to page with full application (and link to apply). If not present, the button will not be shown
 </t>
-        </r>
       </text>
     </comment>
-    <comment ref="G1" authorId="4" xr:uid="{803435A0-8165-0344-9437-CCA1C17B6D10}">
+    <comment ref="G1" authorId="4" shapeId="0" xr:uid="{803435A0-8165-0344-9437-CCA1C17B6D10}">
       <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">Pizzi, Giovanni:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <rFont val="Tahoma"/>
-          </rPr>
-          <t xml:space="preserve">
-When the date is in the past, the job ad will not be shown.
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    When the date is in the past, the job ad will not be shown.
 Not required if the link is not yet present
 </t>
-        </r>
       </text>
     </comment>
   </commentList>
@@ -137,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="131">
   <si>
     <t>Role</t>
   </si>
@@ -148,7 +92,7 @@
     <t>Project</t>
   </si>
   <si>
-    <t xml:space="preserve">Responsible PI</t>
+    <t>Responsible PI</t>
   </si>
   <si>
     <t>Position</t>
@@ -163,13 +107,13 @@
     <t>Comments</t>
   </si>
   <si>
-    <t xml:space="preserve">Scientific and Organizational Coordinator</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paul Scherrer Institute PSI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Klaus Kirch</t>
+    <t>Scientific and Organizational Coordinator</t>
+  </si>
+  <si>
+    <t>Paul Scherrer Institute PSI</t>
+  </si>
+  <si>
+    <t>Klaus Kirch</t>
   </si>
   <si>
     <t xml:space="preserve">Coordination of Muoniverse in close collaboration with the directors </t>
@@ -181,52 +125,52 @@
     <t>Closed</t>
   </si>
   <si>
-    <t xml:space="preserve">Muoniverse Office Assistant</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Support of the consortium, the coordinator and the directors</t>
+    <t>Muoniverse Office Assistant</t>
+  </si>
+  <si>
+    <t>Support of the consortium, the coordinator and the directors</t>
   </si>
   <si>
     <t>https://www.psi.ch/de/hr/stellenangebote/74283-assistentin-50-100</t>
   </si>
   <si>
-    <t xml:space="preserve">Technical Scientific Staff Member</t>
-  </si>
-  <si>
-    <t xml:space="preserve">University of Zurich</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marc Janoschek (UZH), Fabian Natterer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Managing the Quantum Sensing Platform (QSP) for Muoniverse at the Department of Physics at University of Zurich</t>
+    <t>Technical Scientific Staff Member</t>
+  </si>
+  <si>
+    <t>University of Zurich</t>
+  </si>
+  <si>
+    <t>Marc Janoschek (UZH), Fabian Natterer</t>
+  </si>
+  <si>
+    <t>Managing the Quantum Sensing Platform (QSP) for Muoniverse at the Department of Physics at University of Zurich</t>
   </si>
   <si>
     <t>https://apply.mnf.uzh.ch/positiondetails/54984704</t>
   </si>
   <si>
-    <t xml:space="preserve">PhD Student</t>
+    <t>PhD Student</t>
   </si>
   <si>
     <t>T7</t>
   </si>
   <si>
-    <t xml:space="preserve">Giovanni Pizzi (PSI), Nicola Spaldin (ETHZ)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quantum-mechanical simulations of muons in materials</t>
+    <t>Giovanni Pizzi (PSI), Nicola Spaldin (ETHZ)</t>
+  </si>
+  <si>
+    <t>Quantum-mechanical simulations of muons in materials</t>
   </si>
   <si>
     <t>F1,T7</t>
   </si>
   <si>
-    <t xml:space="preserve">Titus Neupert</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Theory for muon sensing of superconductors</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(position already filled)</t>
+    <t>Titus Neupert</t>
+  </si>
+  <si>
+    <t>Theory for muon sensing of superconductors</t>
+  </si>
+  <si>
+    <t>(position already filled)</t>
   </si>
   <si>
     <t>Empa</t>
@@ -235,37 +179,37 @@
     <t>A3</t>
   </si>
   <si>
-    <t xml:space="preserve">Arndt Remhof</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Muon spectroscopy for battery applications</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PhD student</t>
+    <t>Arndt Remhof</t>
+  </si>
+  <si>
+    <t>Muon spectroscopy for battery applications</t>
+  </si>
+  <si>
+    <t>PhD student</t>
   </si>
   <si>
     <t>PSI</t>
   </si>
   <si>
-    <t xml:space="preserve">Sigita Trabesinger</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Already filled</t>
+    <t>Sigita Trabesinger</t>
+  </si>
+  <si>
+    <t>Already filled</t>
   </si>
   <si>
     <t>Postdoc</t>
   </si>
   <si>
-    <t xml:space="preserve">University of Fribourg</t>
+    <t>University of Fribourg</t>
   </si>
   <si>
     <t>F2</t>
   </si>
   <si>
-    <t xml:space="preserve">Christian Bernhard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Low-energy muon spin rotation studies of magnetic and superconducting oxide heterostructures</t>
+    <t>Christian Bernhard</t>
+  </si>
+  <si>
+    <t>Low-energy muon spin rotation studies of magnetic and superconducting oxide heterostructures</t>
   </si>
   <si>
     <t>https://www.unifr.ch/phys/en/department/jobs/</t>
@@ -274,25 +218,25 @@
     <t>F3</t>
   </si>
   <si>
-    <t xml:space="preserve">Zaher Salman</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hybrid interfaces of quantum materials</t>
+    <t>Zaher Salman</t>
+  </si>
+  <si>
+    <t>Hybrid interfaces of quantum materials</t>
   </si>
   <si>
     <t>T4</t>
   </si>
   <si>
-    <t xml:space="preserve">Advanced muon spin spectroscopy</t>
+    <t>Advanced muon spin spectroscopy</t>
   </si>
   <si>
     <t>F6</t>
   </si>
   <si>
-    <t xml:space="preserve">Laura Baudis (UZH), Andreas Knecht (PSI)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ordinary muon capture for neutrinoless double beta decay</t>
+    <t>Laura Baudis (UZH), Andreas Knecht (PSI)</t>
+  </si>
+  <si>
+    <t>Ordinary muon capture for neutrinoless double beta decay</t>
   </si>
   <si>
     <t>https://www.physik.uzh.ch/en/groups/baudis/Positions.html</t>
@@ -301,19 +245,19 @@
     <t>F4</t>
   </si>
   <si>
-    <t xml:space="preserve">Angela Papa (PSI)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hunting for rare muon observables with the muEDM and Mu3e apparatus</t>
+    <t>Angela Papa (PSI)</t>
+  </si>
+  <si>
+    <t>Hunting for rare muon observables with the muEDM and Mu3e apparatus</t>
   </si>
   <si>
     <t>T6</t>
   </si>
   <si>
-    <t xml:space="preserve">H. Luetkens (PSI), M. Janoschek (PSI,UZH), R. Khansanov (PSI)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Development of μSR pressure cells for quantum materials research</t>
+    <t>H. Luetkens (PSI), M. Janoschek (PSI,UZH), R. Khansanov (PSI)</t>
+  </si>
+  <si>
+    <t>Development of μSR pressure cells for quantum materials research</t>
   </si>
   <si>
     <t>https://www.psi.ch/en/hr/job-opportunities/74376-postdoctoral-fellow-in-experimental-physics</t>
@@ -322,7 +266,7 @@
     <t>T6,F1</t>
   </si>
   <si>
-    <t xml:space="preserve">Zurab Guguchia (PSI)</t>
+    <t>Zurab Guguchia (PSI)</t>
   </si>
   <si>
     <t xml:space="preserve">Uniaxial and hydrostatic pressure studies on quantum materials </t>
@@ -337,10 +281,10 @@
     <t>T2</t>
   </si>
   <si>
-    <t xml:space="preserve">T. Pieloni (EPFL), A. Lombardi (CERN), M. Seidel (PSI,EPFL)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Acceleration of an ultra-low-emittance mu+ beam</t>
+    <t>T. Pieloni (EPFL), A. Lombardi (CERN), M. Seidel (PSI,EPFL)</t>
+  </si>
+  <si>
+    <t>Acceleration of an ultra-low-emittance mu+ beam</t>
   </si>
   <si>
     <t>https://careers.epfl.ch/job/Lausanne-PhD-Laboratory-of-Particle-Accelerator-Physics-%28LPAP%29/1164210555/</t>
@@ -352,91 +296,91 @@
     <t>A1</t>
   </si>
   <si>
-    <t xml:space="preserve">U. Grossner</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Defect characterization for advanced power semiconductor devices</t>
-  </si>
-  <si>
-    <t xml:space="preserve">University of Geneva</t>
+    <t>U. Grossner</t>
+  </si>
+  <si>
+    <t>Defect characterization for advanced power semiconductor devices</t>
+  </si>
+  <si>
+    <t>University of Geneva</t>
   </si>
   <si>
     <t>F3,F7</t>
   </si>
   <si>
-    <t xml:space="preserve">M. Kowalska (CERN)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Upgrades to the polarisation beamline at ISOLDE-CERN for material science and magnetisation radii studies</t>
-  </si>
-  <si>
-    <t xml:space="preserve">internal candidate</t>
+    <t>M. Kowalska (CERN)</t>
+  </si>
+  <si>
+    <t>Upgrades to the polarisation beamline at ISOLDE-CERN for material science and magnetisation radii studies</t>
+  </si>
+  <si>
+    <t>internal candidate</t>
   </si>
   <si>
     <t>F1</t>
   </si>
   <si>
-    <t xml:space="preserve">Zurab Guguchia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Establishing Muon Spin Fingerprints of Intrinsic Time-Reversal Symmetry-Breaking Superconducting and Normal States</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fabian von Rohr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Advanced Synthesis Methods of Quantum Materials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">University of Zürich</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fabian Natterer (UZH)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hunting for hints for time-reversal symmetry-breaking superconductivity in Josephosn Junction STM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">internal candidate, start 1. September 2026</t>
+    <t>Zurab Guguchia</t>
+  </si>
+  <si>
+    <t>Establishing Muon Spin Fingerprints of Intrinsic Time-Reversal Symmetry-Breaking Superconducting and Normal States</t>
+  </si>
+  <si>
+    <t>Fabian von Rohr</t>
+  </si>
+  <si>
+    <t>Advanced Synthesis Methods of Quantum Materials</t>
+  </si>
+  <si>
+    <t>University of Zürich</t>
+  </si>
+  <si>
+    <t>Fabian Natterer (UZH)</t>
+  </si>
+  <si>
+    <t>Hunting for hints for time-reversal symmetry-breaking superconductivity in Josephosn Junction STM</t>
+  </si>
+  <si>
+    <t>internal candidate, start 1. September 2026</t>
   </si>
   <si>
     <t>T1</t>
   </si>
   <si>
-    <t xml:space="preserve">Aldo Antognini</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Development of a micro-beam of positive muons for particle, atomic and solid state physics</t>
+    <t>Aldo Antognini</t>
+  </si>
+  <si>
+    <t>Development of a micro-beam of positive muons for particle, atomic and solid state physics</t>
   </si>
   <si>
     <t>A4</t>
   </si>
   <si>
-    <t xml:space="preserve">Aldo Antognini (PSI), Anna Soter (ETHZ)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Development of a laser system (thin-disk laser followed by OPO) for pump and probe muSR studies</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paul Scherrer Institut PSI / SNM</t>
+    <t>Aldo Antognini (PSI), Anna Soter (ETHZ)</t>
+  </si>
+  <si>
+    <t>Development of a laser system (thin-disk laser followed by OPO) for pump and probe muSR studies</t>
+  </si>
+  <si>
+    <t>Paul Scherrer Institut PSI / SNM</t>
   </si>
   <si>
     <t>A5</t>
   </si>
   <si>
-    <t xml:space="preserve">Michael Heiss</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Non-destructive elemental analysis of archaeological and cultural heritage artefacts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Swiss National Museum SNM / PSI</t>
+    <t>Michael Heiss</t>
+  </si>
+  <si>
+    <t>Non-destructive elemental analysis of archaeological and cultural heritage artefacts</t>
+  </si>
+  <si>
+    <t>Swiss National Museum SNM / PSI</t>
   </si>
   <si>
     <t>MuseumPlatform</t>
   </si>
   <si>
-    <t xml:space="preserve">Katharina Schmidt-Ott</t>
+    <t>Katharina Schmidt-Ott</t>
   </si>
   <si>
     <t>https://www.nationalmuseum.ch/de/jobs/postdoktorand-in-muoniverse-museum-platform-software-fur-die-mixe-datenanalyse-100-befristet-bis-30-april-2030-46138</t>
@@ -448,19 +392,19 @@
     <t xml:space="preserve">Muon beams and fundamental atomic, nuclear and particle physics </t>
   </si>
   <si>
-    <t xml:space="preserve">part of PSI's director relief effort</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Postdoc/Software Engineer</t>
+    <t>part of PSI's director relief effort</t>
+  </si>
+  <si>
+    <t>Postdoc/Software Engineer</t>
   </si>
   <si>
     <t>OpenScience</t>
   </si>
   <si>
-    <t xml:space="preserve">Giovanni Pizzi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Design of a secure data sharing portal for muon data</t>
+    <t>Giovanni Pizzi</t>
+  </si>
+  <si>
+    <t>Design of a secure data sharing portal for muon data</t>
   </si>
   <si>
     <t>F5</t>
@@ -469,105 +413,105 @@
     <t xml:space="preserve">Paolo Crivelli </t>
   </si>
   <si>
-    <t xml:space="preserve">Muonium spectroscopy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">potential internal candidate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Peter Stoffer (PSI and UZH)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Advancing the theoretical framework for rare muon observables</t>
+    <t>Muonium spectroscopy</t>
+  </si>
+  <si>
+    <t>potential internal candidate</t>
+  </si>
+  <si>
+    <t>Peter Stoffer (PSI and UZH)</t>
+  </si>
+  <si>
+    <t>Advancing the theoretical framework for rare muon observables</t>
   </si>
   <si>
     <t>T5</t>
   </si>
   <si>
-    <t xml:space="preserve">Cryogenic detector to accurately track positrons from muon decays</t>
+    <t>Cryogenic detector to accurately track positrons from muon decays</t>
   </si>
   <si>
     <t>F7</t>
   </si>
   <si>
-    <t xml:space="preserve">Andreas Knecht (PSI)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">High-precision muonic x-ray measurements of low-Z elements with a metallic magnetic calorimeter</t>
+    <t>Andreas Knecht (PSI)</t>
+  </si>
+  <si>
+    <t>High-precision muonic x-ray measurements of low-Z elements with a metallic magnetic calorimeter</t>
   </si>
   <si>
     <t>https://www.psi.ch/en/hr/job-opportunities/74339-postdoctoral-fellow-in-muon-physics</t>
   </si>
   <si>
-    <t xml:space="preserve">Johanna Nordlander (UZH)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thin-film synthesis and muon spectroscopy for novel oxide quantum materials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Philipp Schmidt-Wellenburg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exploiting pixelated silicon detectors for the search of the electric dipole moment of the muon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">For any job offering, please add a row filling *all* columns</t>
+    <t>Johanna Nordlander (UZH)</t>
+  </si>
+  <si>
+    <t>Thin-film synthesis and muon spectroscopy for novel oxide quantum materials</t>
+  </si>
+  <si>
+    <t>Philipp Schmidt-Wellenburg</t>
+  </si>
+  <si>
+    <t>Exploiting pixelated silicon detectors for the search of the electric dipole moment of the muon</t>
+  </si>
+  <si>
+    <t>For any job offering, please add a row filling *all* columns</t>
   </si>
   <si>
     <t>Notes:</t>
   </si>
   <si>
-    <t xml:space="preserve">- try to use a consistent naming for job position and location (institution name)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- try to be as concise as possible in the position description</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- ensure you have the direct URL to the correct advertisement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- deadline might not be shown on the muoniverse.ch website to avoid making it complex to keep things udpated, but it's important to put as it can be used to remove openings from the website once they are expired</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOTE: at the moment, the content of this file is NOT automatically mirrored to the website! You need to ask someone with permissions to apply the changes and put them online</t>
+    <t>- try to use a consistent naming for job position and location (institution name)</t>
+  </si>
+  <si>
+    <t>- try to be as concise as possible in the position description</t>
+  </si>
+  <si>
+    <t>- ensure you have the direct URL to the correct advertisement</t>
+  </si>
+  <si>
+    <t>- deadline might not be shown on the muoniverse.ch website to avoid making it complex to keep things udpated, but it's important to put as it can be used to remove openings from the website once they are expired</t>
+  </si>
+  <si>
+    <t>NOTE: at the moment, the content of this file is NOT automatically mirrored to the website! You need to ask someone with permissions to apply the changes and put them online</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
-      <sz val="12.000000"/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
     <font>
       <u/>
-      <sz val="12.000000"/>
+      <sz val="12"/>
       <color theme="10"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="12.000000"/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
     <font>
       <u/>
-      <sz val="12.000000"/>
+      <sz val="12"/>
       <color theme="10"/>
       <name val="Aptos Narrow"/>
     </font>
     <font>
-      <sz val="12.000000"/>
+      <sz val="12"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -581,42 +525,39 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
       </patternFill>
     </fill>
   </fills>
   <borders count="1">
     <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="2">
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1"/>
-    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf fontId="2" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
-      <protection hidden="0" locked="1"/>
-    </xf>
-    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+  <cellXfs count="11">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf fontId="4" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="4" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="1" applyFont="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" quotePrefix="1"/>
-    <xf fontId="2" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -637,296 +578,13 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="Pizzi, Giovanni" id="{6922F27C-BE0C-7399-14F1-F78F015972B1}" userId="S::giovanni.pizzi@psi.ch::fcd49011-dac4-4c01-9bc6-eefdd0021243" providerId="AD"/>
-  <person displayName="Pizzi, Giovanni" id="{DC79B204-8000-E0C1-D3CC-5CF54A964D2F}" userId="S::giovanni.pizzi@psi.ch::fcd49011-dac4-4c01-9bc6-eefdd0021243" providerId="Teamlab"/>
+  <person displayName="Pizzi, Giovanni" id="{EBDA578D-3C72-B747-71F1-C7EA0ED4AB5E}" userId="S::giovanni.pizzi@psi.ch::fcd49011-dac4-4c01-9bc6-eefdd0021243" providerId="AD"/>
+  <person displayName="Pizzi, Giovanni" id="{B8D38DFC-CDC3-CB12-E96C-36BC521976DC}" userId="S::giovanni.pizzi@psi.ch::fcd49011-dac4-4c01-9bc6-eefdd0021243" providerId="Teamlab"/>
 </personList>
 </file>
 
-<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="1F497D"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="EEECE1"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="4F81BD"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="C0504D"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="9BBB59"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="8064A2"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="4BACC6"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="F79646"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0000FF"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="800080"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Angsana New"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Cordia New"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme name="Office">
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="40000">
-              <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-</a:theme>
-</file>
-
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1149,28 +807,29 @@
       </a:style>
     </a:lnDef>
   </a:objectDefaults>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="A1" dT="2026-02-02T10:18:20.32Z" personId="{6922F27C-BE0C-7399-14F1-F78F015972B1}" id="{D3909E3A-CF3A-6144-B66D-EC5AECD54804}" done="0">
+  <threadedComment ref="A1" dT="2026-02-02T10:18:20.32" personId="{EBDA578D-3C72-B747-71F1-C7EA0ED4AB5E}" id="{D3909E3A-CF3A-6144-B66D-EC5AECD54804}">
     <text xml:space="preserve">Please use standardized phrasing (copy from lines above, if needed)
 </text>
   </threadedComment>
-  <threadedComment ref="B1" dT="2026-02-02T10:18:52.37Z" personId="{6922F27C-BE0C-7399-14F1-F78F015972B1}" id="{3A2C8F42-915E-4B42-8C35-1087C2FD6E67}" done="0">
+  <threadedComment ref="B1" dT="2026-02-02T10:18:52.37" personId="{EBDA578D-3C72-B747-71F1-C7EA0ED4AB5E}" id="{3A2C8F42-915E-4B42-8C35-1087C2FD6E67}">
     <text xml:space="preserve">Please use standardized name (copy name from rows above, if one already exists)
 </text>
   </threadedComment>
-  <threadedComment ref="E1" dT="2026-02-02T10:19:08.34Z" personId="{DC79B204-8000-E0C1-D3CC-5CF54A964D2F}" id="{0DD1F034-F3C2-6143-B5EE-4D8ACB9B94D3}" done="0">
+  <threadedComment ref="E1" dT="2026-02-02T10:19:08.34" personId="{B8D38DFC-CDC3-CB12-E96C-36BC521976DC}" id="{0DD1F034-F3C2-6143-B5EE-4D8ACB9B94D3}">
     <text xml:space="preserve">Short 1-line job description
 </text>
   </threadedComment>
-  <threadedComment ref="F1" dT="2026-02-02T10:19:37.74Z" personId="{DC79B204-8000-E0C1-D3CC-5CF54A964D2F}" id="{7B781CE5-788D-EE45-89AA-868478A6290E}" done="0">
+  <threadedComment ref="F1" dT="2026-02-02T10:19:37.74" personId="{B8D38DFC-CDC3-CB12-E96C-36BC521976DC}" id="{7B781CE5-788D-EE45-89AA-868478A6290E}">
     <text xml:space="preserve">Direct link to page with full application (and link to apply). If not present, the button will not be shown
 </text>
   </threadedComment>
-  <threadedComment ref="G1" dT="2026-02-05T22:35:50.45Z" personId="{DC79B204-8000-E0C1-D3CC-5CF54A964D2F}" id="{803435A0-8165-0344-9437-CCA1C17B6D10}" done="0">
+  <threadedComment ref="G1" dT="2026-02-05T22:35:50.45" personId="{B8D38DFC-CDC3-CB12-E96C-36BC521976DC}" id="{803435A0-8165-0344-9437-CCA1C17B6D10}">
     <text xml:space="preserve">When the date is in the past, the job ad will not be shown.
 Not required if the link is not yet present
 </text>
@@ -1179,20 +838,21 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:H34"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="77.77734375"/>
-    <col bestFit="1" customWidth="1" min="2" max="2" width="28.50390625"/>
-    <col customWidth="1" min="3" max="3" width="29.21484375"/>
-    <col customWidth="1" min="4" max="4" width="52.21484375"/>
-    <col customWidth="1" min="5" max="5" width="81.33203125"/>
-    <col customWidth="1" min="6" max="6" width="57.5546875"/>
-    <col customWidth="1" min="7" max="7" style="1" width="16.6640625"/>
-    <col bestFit="1" customWidth="1" min="8" max="8" width="44.83203125"/>
+    <col min="1" max="1" width="37.5" customWidth="1"/>
+    <col min="2" max="2" width="28.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.1640625" customWidth="1"/>
+    <col min="4" max="4" width="52.1640625" customWidth="1"/>
+    <col min="5" max="5" width="81.33203125" customWidth="1"/>
+    <col min="6" max="6" width="57.5" customWidth="1"/>
+    <col min="7" max="7" width="16.6640625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="44.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1218,75 +878,74 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="4" t="s">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" s="4" t="s">
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="4" t="s">
         <v>12</v>
       </c>
       <c r="G2" s="1">
         <v>46101</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" s="0" customFormat="1">
-      <c r="A3" s="4" t="s">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="4" t="s">
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="5" t="s">
         <v>16</v>
       </c>
       <c r="G3" s="1">
         <v>46142</v>
       </c>
     </row>
-    <row r="4" s="0" customFormat="1">
-      <c r="A4" s="4" t="s">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" t="s">
         <v>20</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="G4" s="1"/>
-    </row>
-    <row r="5">
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>22</v>
       </c>
       <c r="B5" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" t="s">
         <v>23</v>
       </c>
       <c r="D5" t="s">
@@ -1296,14 +955,14 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" ht="15">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>22</v>
       </c>
       <c r="B6" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" t="s">
         <v>26</v>
       </c>
       <c r="D6" t="s">
@@ -1319,14 +978,14 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" ht="15">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>22</v>
       </c>
       <c r="B7" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" t="s">
         <v>31</v>
       </c>
       <c r="D7" t="s">
@@ -1336,17 +995,17 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" ht="15">
-      <c r="A8" s="4" t="s">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
         <v>34</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" t="s">
         <v>35</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" t="s">
         <v>31</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" t="s">
         <v>36</v>
       </c>
       <c r="E8" t="s">
@@ -1359,27 +1018,33 @@
         <v>37</v>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1">
+    <row r="9" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>38</v>
       </c>
       <c r="B9" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" t="s">
         <v>40</v>
       </c>
       <c r="D9" t="s">
         <v>41</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="F9" s="4" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="10" ht="15">
+      <c r="G9" s="1">
+        <v>46113</v>
+      </c>
+      <c r="H9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1396,27 +1061,27 @@
         <v>46</v>
       </c>
     </row>
-    <row r="11" ht="15">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C11" s="5" t="s">
+      <c r="B11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" t="s">
         <v>47</v>
       </c>
       <c r="D11" t="s">
         <v>45</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" t="s">
         <v>48</v>
       </c>
       <c r="H11" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="12" ht="15">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>22</v>
       </c>
@@ -1432,11 +1097,11 @@
       <c r="E12" t="s">
         <v>51</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="5" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="13" ht="15">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -1449,15 +1114,15 @@
       <c r="D13" t="s">
         <v>54</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="E13" s="6" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="14" ht="15">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>38</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" t="s">
         <v>9</v>
       </c>
       <c r="C14" t="s">
@@ -1466,14 +1131,14 @@
       <c r="D14" t="s">
         <v>57</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="5" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="15" ht="15">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>22</v>
       </c>
@@ -1486,14 +1151,14 @@
       <c r="D15" t="s">
         <v>61</v>
       </c>
-      <c r="E15" s="8" t="s">
+      <c r="E15" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="F15" s="5" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="16" ht="15">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -1506,17 +1171,17 @@
       <c r="D16" t="s">
         <v>66</v>
       </c>
-      <c r="E16" s="9" t="s">
+      <c r="E16" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="F16" s="5" t="s">
         <v>68</v>
       </c>
       <c r="G16" s="1">
         <v>46127</v>
       </c>
     </row>
-    <row r="17" ht="15">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>22</v>
       </c>
@@ -1533,7 +1198,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="18" ht="15">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>38</v>
       </c>
@@ -1556,11 +1221,11 @@
         <v>77</v>
       </c>
     </row>
-    <row r="19" ht="15">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>22</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" t="s">
         <v>9</v>
       </c>
       <c r="C19" t="s">
@@ -1569,15 +1234,15 @@
       <c r="D19" t="s">
         <v>79</v>
       </c>
-      <c r="E19" s="5" t="s">
+      <c r="E19" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="20" ht="15">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>22</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" t="s">
         <v>73</v>
       </c>
       <c r="C20" t="s">
@@ -1586,16 +1251,15 @@
       <c r="D20" t="s">
         <v>81</v>
       </c>
-      <c r="E20" s="5" t="s">
+      <c r="E20" t="s">
         <v>82</v>
       </c>
-      <c r="G20" s="1"/>
-    </row>
-    <row r="21" ht="15">
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>22</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" t="s">
         <v>83</v>
       </c>
       <c r="C21" t="s">
@@ -1604,7 +1268,7 @@
       <c r="D21" t="s">
         <v>84</v>
       </c>
-      <c r="E21" s="5" t="s">
+      <c r="E21" t="s">
         <v>85</v>
       </c>
       <c r="G21" s="1">
@@ -1614,11 +1278,11 @@
         <v>86</v>
       </c>
     </row>
-    <row r="22" ht="15">
-      <c r="A22" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B22" s="5" t="s">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>22</v>
+      </c>
+      <c r="B22" t="s">
         <v>9</v>
       </c>
       <c r="C22" t="s">
@@ -1627,15 +1291,15 @@
       <c r="D22" t="s">
         <v>88</v>
       </c>
-      <c r="E22" s="5" t="s">
+      <c r="E22" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="23" ht="15">
-      <c r="A23" s="5" t="s">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
         <v>38</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" t="s">
         <v>9</v>
       </c>
       <c r="C23" t="s">
@@ -1644,32 +1308,32 @@
       <c r="D23" t="s">
         <v>88</v>
       </c>
-      <c r="E23" s="5" t="s">
+      <c r="E23" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="24" ht="15">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>38</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" t="s">
         <v>9</v>
       </c>
       <c r="C24" t="s">
         <v>90</v>
       </c>
-      <c r="D24" s="5" t="s">
+      <c r="D24" t="s">
         <v>91</v>
       </c>
       <c r="E24" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="25" ht="15">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>22</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" t="s">
         <v>93</v>
       </c>
       <c r="C25" t="s">
@@ -1678,11 +1342,11 @@
       <c r="D25" t="s">
         <v>95</v>
       </c>
-      <c r="E25" s="4" t="s">
+      <c r="E25" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="26" ht="15">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>38</v>
       </c>
@@ -1695,21 +1359,21 @@
       <c r="D26" t="s">
         <v>99</v>
       </c>
-      <c r="E26" s="4" t="s">
+      <c r="E26" t="s">
         <v>96</v>
       </c>
-      <c r="F26" s="7" t="s">
+      <c r="F26" s="5" t="s">
         <v>100</v>
       </c>
       <c r="G26" s="1">
         <v>46111</v>
       </c>
     </row>
-    <row r="27" ht="15">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>38</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="B27" t="s">
         <v>9</v>
       </c>
       <c r="C27" t="s">
@@ -1718,21 +1382,21 @@
       <c r="D27" t="s">
         <v>10</v>
       </c>
-      <c r="E27" s="4" t="s">
+      <c r="E27" t="s">
         <v>102</v>
       </c>
       <c r="H27" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="28" ht="15">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>104</v>
       </c>
       <c r="B28" t="s">
         <v>9</v>
       </c>
-      <c r="C28" s="4" t="s">
+      <c r="C28" t="s">
         <v>105</v>
       </c>
       <c r="D28" t="s">
@@ -1741,10 +1405,9 @@
       <c r="E28" t="s">
         <v>107</v>
       </c>
-      <c r="F28" s="10"/>
-      <c r="G28" s="1"/>
-    </row>
-    <row r="29" ht="15">
+      <c r="F28" s="8"/>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>22</v>
       </c>
@@ -1760,11 +1423,11 @@
       <c r="E29" t="s">
         <v>110</v>
       </c>
-      <c r="H29" s="5" t="s">
+      <c r="H29" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="30" ht="15">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>22</v>
       </c>
@@ -1781,7 +1444,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="31" ht="15">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>38</v>
       </c>
@@ -1798,11 +1461,11 @@
         <v>115</v>
       </c>
     </row>
-    <row r="32" ht="15">
-      <c r="A32" s="5" t="s">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
         <v>38</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="B32" t="s">
         <v>9</v>
       </c>
       <c r="C32" t="s">
@@ -1814,11 +1477,11 @@
       <c r="E32" t="s">
         <v>118</v>
       </c>
-      <c r="F32" s="7" t="s">
+      <c r="F32" s="5" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="33" ht="15">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>22</v>
       </c>
@@ -1835,7 +1498,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="34" ht="15">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>22</v>
       </c>
@@ -1852,74 +1515,70 @@
         <v>123</v>
       </c>
     </row>
-    <row r="35" ht="15"/>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="F2" tooltip=""/>
-    <hyperlink r:id="rId2" ref="F3"/>
-    <hyperlink r:id="rId3" ref="F4"/>
-    <hyperlink r:id="rId4" ref="F9" tooltip="https://www.unifr.ch/phys/en/department/jobs/"/>
-    <hyperlink r:id="rId5" ref="F12"/>
-    <hyperlink r:id="rId6" ref="F14"/>
-    <hyperlink r:id="rId7" ref="F15"/>
-    <hyperlink r:id="rId8" ref="F16"/>
-    <hyperlink r:id="rId9" ref="F26"/>
-    <hyperlink r:id="rId10" ref="F32"/>
+    <hyperlink ref="F2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="F3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="F4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="F9" r:id="rId4" tooltip="https://www.unifr.ch/phys/en/department/jobs/" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="F12" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="F14" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="F15" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="F16" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="F26" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="F32" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
   </hyperlinks>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="0" verticalDpi="0" copies="1"/>
-  <headerFooter/>
-  <legacyDrawing r:id="rId13"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <legacyDrawing r:id="rId11"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:A9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="175.1640625"/>
+    <col min="1" max="1" width="175.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="11" t="s">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A4" s="9" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="11" t="s">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A5" s="9" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="11" t="s">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A6" s="9" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="11" t="s">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A7" s="9" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="12" t="s">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A9" s="10" t="s">
         <v>130</v>
       </c>
     </row>
   </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Adding one job link
</commit_message>
<xml_diff>
--- a/job-openings-scripts/muoniverse-job-openings.xlsx
+++ b/job-openings-scripts/muoniverse-job-openings.xlsx
@@ -137,7 +137,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="142">
   <si>
     <t>Role</t>
   </si>
@@ -533,6 +533,9 @@
   </si>
   <si>
     <t xml:space="preserve">Thin-film synthesis and muon spectroscopy for novel oxide quantum materials</t>
+  </si>
+  <si>
+    <t>https://www.physik.uzh.ch/en/groups/nordlander/Positions.html</t>
   </si>
   <si>
     <t xml:space="preserve">Philipp Schmidt-Wellenburg</t>
@@ -667,8 +670,8 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="Pizzi, Giovanni" id="{448E3ADC-194E-5EFE-7B22-885263FF50D4}" userId="S::giovanni.pizzi@psi.ch::fcd49011-dac4-4c01-9bc6-eefdd0021243" providerId="AD"/>
-  <person displayName="Pizzi, Giovanni" id="{0E0B45BC-7DEA-D6DE-3E48-0C8CF6DD35C5}" userId="S::giovanni.pizzi@psi.ch::fcd49011-dac4-4c01-9bc6-eefdd0021243" providerId="Teamlab"/>
+  <person displayName="Pizzi, Giovanni" id="{830FAB3A-DC8D-0A27-C883-C73EE7A2E43A}" userId="S::giovanni.pizzi@psi.ch::fcd49011-dac4-4c01-9bc6-eefdd0021243" providerId="AD"/>
+  <person displayName="Pizzi, Giovanni" id="{7607B40F-3534-1C29-FDB0-6304E4AD4A1B}" userId="S::giovanni.pizzi@psi.ch::fcd49011-dac4-4c01-9bc6-eefdd0021243" providerId="Teamlab"/>
 </personList>
 </file>
 
@@ -1184,23 +1187,23 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="A1" dT="2026-02-02T10:18:20.32Z" personId="{448E3ADC-194E-5EFE-7B22-885263FF50D4}" id="{D3909E3A-CF3A-6144-B66D-EC5AECD54804}" done="0">
+  <threadedComment ref="A1" dT="2026-02-02T10:18:20.32Z" personId="{830FAB3A-DC8D-0A27-C883-C73EE7A2E43A}" id="{D3909E3A-CF3A-6144-B66D-EC5AECD54804}" done="0">
     <text xml:space="preserve">Please use standardized phrasing (copy from lines above, if needed)
 </text>
   </threadedComment>
-  <threadedComment ref="B1" dT="2026-02-02T10:18:52.37Z" personId="{448E3ADC-194E-5EFE-7B22-885263FF50D4}" id="{3A2C8F42-915E-4B42-8C35-1087C2FD6E67}" done="0">
+  <threadedComment ref="B1" dT="2026-02-02T10:18:52.37Z" personId="{830FAB3A-DC8D-0A27-C883-C73EE7A2E43A}" id="{3A2C8F42-915E-4B42-8C35-1087C2FD6E67}" done="0">
     <text xml:space="preserve">Please use standardized name (copy name from rows above, if one already exists)
 </text>
   </threadedComment>
-  <threadedComment ref="E1" dT="2026-02-02T10:19:08.34Z" personId="{0E0B45BC-7DEA-D6DE-3E48-0C8CF6DD35C5}" id="{0DD1F034-F3C2-6143-B5EE-4D8ACB9B94D3}" done="0">
+  <threadedComment ref="E1" dT="2026-02-02T10:19:08.34Z" personId="{7607B40F-3534-1C29-FDB0-6304E4AD4A1B}" id="{0DD1F034-F3C2-6143-B5EE-4D8ACB9B94D3}" done="0">
     <text xml:space="preserve">Short 1-line job description
 </text>
   </threadedComment>
-  <threadedComment ref="F1" dT="2026-02-02T10:19:37.74Z" personId="{0E0B45BC-7DEA-D6DE-3E48-0C8CF6DD35C5}" id="{7B781CE5-788D-EE45-89AA-868478A6290E}" done="0">
+  <threadedComment ref="F1" dT="2026-02-02T10:19:37.74Z" personId="{7607B40F-3534-1C29-FDB0-6304E4AD4A1B}" id="{7B781CE5-788D-EE45-89AA-868478A6290E}" done="0">
     <text xml:space="preserve">Direct link to page with full application (and link to apply). If not present, the button will not be shown
 </text>
   </threadedComment>
-  <threadedComment ref="G1" dT="2026-02-05T22:35:50.45Z" personId="{0E0B45BC-7DEA-D6DE-3E48-0C8CF6DD35C5}" id="{803435A0-8165-0344-9437-CCA1C17B6D10}" done="0">
+  <threadedComment ref="G1" dT="2026-02-05T22:35:50.45Z" personId="{7607B40F-3534-1C29-FDB0-6304E4AD4A1B}" id="{803435A0-8165-0344-9437-CCA1C17B6D10}" done="0">
     <text xml:space="preserve">When the date is in the past, the job ad will not be shown.
 Not required if the link is not yet present
 </text>
@@ -1917,6 +1920,9 @@
       <c r="E34" t="s">
         <v>131</v>
       </c>
+      <c r="F34" s="7" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="35" ht="15">
       <c r="A35" t="s">
@@ -1929,10 +1935,10 @@
         <v>53</v>
       </c>
       <c r="D35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E35" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="36" ht="15">
@@ -1959,12 +1965,13 @@
     <hyperlink r:id="rId13" ref="F31"/>
     <hyperlink r:id="rId14" ref="F32"/>
     <hyperlink r:id="rId15" ref="F33"/>
+    <hyperlink r:id="rId16" ref="F34"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="0" verticalDpi="0" copies="1"/>
   <headerFooter/>
-  <legacyDrawing r:id="rId18"/>
+  <legacyDrawing r:id="rId19"/>
 </worksheet>
 </file>
 
@@ -1977,37 +1984,37 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="11" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Closing one position, opening another
</commit_message>
<xml_diff>
--- a/job-openings-scripts/muoniverse-job-openings.xlsx
+++ b/job-openings-scripts/muoniverse-job-openings.xlsx
@@ -137,7 +137,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="143">
   <si>
     <t>Role</t>
   </si>
@@ -230,6 +230,9 @@
   </si>
   <si>
     <t xml:space="preserve">Quantum-mechanical simulations of muons in materials</t>
+  </si>
+  <si>
+    <t>https://www.psi.ch/en/hr/job-opportunities/74609-phd-student-in-quantum-mechanical-simulations-of-muons-in-materials</t>
   </si>
   <si>
     <t>F1,T7</t>
@@ -670,8 +673,8 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="Pizzi, Giovanni" id="{830FAB3A-DC8D-0A27-C883-C73EE7A2E43A}" userId="S::giovanni.pizzi@psi.ch::fcd49011-dac4-4c01-9bc6-eefdd0021243" providerId="AD"/>
-  <person displayName="Pizzi, Giovanni" id="{7607B40F-3534-1C29-FDB0-6304E4AD4A1B}" userId="S::giovanni.pizzi@psi.ch::fcd49011-dac4-4c01-9bc6-eefdd0021243" providerId="Teamlab"/>
+  <person displayName="Pizzi, Giovanni" id="{8D3C90E1-12D3-28A0-88CF-117F6FC1D327}" userId="S::giovanni.pizzi@psi.ch::fcd49011-dac4-4c01-9bc6-eefdd0021243" providerId="AD"/>
+  <person displayName="Pizzi, Giovanni" id="{8C4FA6FE-6573-C40F-F91D-688FCBB7A930}" userId="S::giovanni.pizzi@psi.ch::fcd49011-dac4-4c01-9bc6-eefdd0021243" providerId="Teamlab"/>
 </personList>
 </file>
 
@@ -1187,23 +1190,23 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="A1" dT="2026-02-02T10:18:20.32Z" personId="{830FAB3A-DC8D-0A27-C883-C73EE7A2E43A}" id="{D3909E3A-CF3A-6144-B66D-EC5AECD54804}" done="0">
+  <threadedComment ref="A1" dT="2026-02-02T10:18:20.32Z" personId="{8D3C90E1-12D3-28A0-88CF-117F6FC1D327}" id="{D3909E3A-CF3A-6144-B66D-EC5AECD54804}" done="0">
     <text xml:space="preserve">Please use standardized phrasing (copy from lines above, if needed)
 </text>
   </threadedComment>
-  <threadedComment ref="B1" dT="2026-02-02T10:18:52.37Z" personId="{830FAB3A-DC8D-0A27-C883-C73EE7A2E43A}" id="{3A2C8F42-915E-4B42-8C35-1087C2FD6E67}" done="0">
+  <threadedComment ref="B1" dT="2026-02-02T10:18:52.37Z" personId="{8D3C90E1-12D3-28A0-88CF-117F6FC1D327}" id="{3A2C8F42-915E-4B42-8C35-1087C2FD6E67}" done="0">
     <text xml:space="preserve">Please use standardized name (copy name from rows above, if one already exists)
 </text>
   </threadedComment>
-  <threadedComment ref="E1" dT="2026-02-02T10:19:08.34Z" personId="{7607B40F-3534-1C29-FDB0-6304E4AD4A1B}" id="{0DD1F034-F3C2-6143-B5EE-4D8ACB9B94D3}" done="0">
+  <threadedComment ref="E1" dT="2026-02-02T10:19:08.34Z" personId="{8C4FA6FE-6573-C40F-F91D-688FCBB7A930}" id="{0DD1F034-F3C2-6143-B5EE-4D8ACB9B94D3}" done="0">
     <text xml:space="preserve">Short 1-line job description
 </text>
   </threadedComment>
-  <threadedComment ref="F1" dT="2026-02-02T10:19:37.74Z" personId="{7607B40F-3534-1C29-FDB0-6304E4AD4A1B}" id="{7B781CE5-788D-EE45-89AA-868478A6290E}" done="0">
+  <threadedComment ref="F1" dT="2026-02-02T10:19:37.74Z" personId="{8C4FA6FE-6573-C40F-F91D-688FCBB7A930}" id="{7B781CE5-788D-EE45-89AA-868478A6290E}" done="0">
     <text xml:space="preserve">Direct link to page with full application (and link to apply). If not present, the button will not be shown
 </text>
   </threadedComment>
-  <threadedComment ref="G1" dT="2026-02-05T22:35:50.45Z" personId="{7607B40F-3534-1C29-FDB0-6304E4AD4A1B}" id="{803435A0-8165-0344-9437-CCA1C17B6D10}" done="0">
+  <threadedComment ref="G1" dT="2026-02-05T22:35:50.45Z" personId="{8C4FA6FE-6573-C40F-F91D-688FCBB7A930}" id="{803435A0-8165-0344-9437-CCA1C17B6D10}" done="0">
     <text xml:space="preserve">When the date is in the past, the job ad will not be shown.
 Not required if the link is not yet present
 </text>
@@ -1352,6 +1355,12 @@
       <c r="E6" t="s">
         <v>30</v>
       </c>
+      <c r="F6" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="G6" s="1">
+        <v>46188</v>
+      </c>
     </row>
     <row r="7" ht="15">
       <c r="A7" t="s">
@@ -1361,19 +1370,19 @@
         <v>23</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G7" s="1">
         <v>46029</v>
       </c>
       <c r="H7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" ht="15">
@@ -1381,59 +1390,59 @@
         <v>27</v>
       </c>
       <c r="B8" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" ht="15">
       <c r="A9" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E9" t="s">
         <v>39</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="E9" t="s">
-        <v>38</v>
       </c>
       <c r="G9" s="1">
         <v>46029</v>
       </c>
       <c r="H9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" ht="16.5" customHeight="1">
       <c r="A10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D10" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G10" s="1">
         <v>46113</v>
@@ -1450,16 +1459,16 @@
         <v>9</v>
       </c>
       <c r="C11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D11" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12" ht="15">
@@ -1470,19 +1479,19 @@
         <v>9</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G12" s="1">
         <v>46113</v>
       </c>
       <c r="H12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="13" ht="15">
@@ -1493,16 +1502,16 @@
         <v>23</v>
       </c>
       <c r="C13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D13" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E13" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="14" ht="15">
@@ -1513,36 +1522,36 @@
         <v>9</v>
       </c>
       <c r="C14" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D14" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="15" ht="15">
       <c r="A15" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C15" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D15" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="16" ht="15">
@@ -1553,16 +1562,16 @@
         <v>9</v>
       </c>
       <c r="C16" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D16" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="17" ht="15">
@@ -1570,19 +1579,19 @@
         <v>27</v>
       </c>
       <c r="B17" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C17" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D17" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G17" s="1">
         <v>46127</v>
@@ -1593,39 +1602,39 @@
         <v>27</v>
       </c>
       <c r="B18" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C18" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E18" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="19" ht="15">
       <c r="A19" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B19" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C19" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D19" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E19" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G19" s="1">
         <v>46143</v>
       </c>
       <c r="H19" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="20" ht="15">
@@ -1636,13 +1645,13 @@
         <v>9</v>
       </c>
       <c r="C20" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D20" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="21" ht="15">
@@ -1650,16 +1659,16 @@
         <v>27</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C21" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D21" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G21" s="1"/>
     </row>
@@ -1668,22 +1677,22 @@
         <v>27</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C22" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D22" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G22" s="1">
         <v>46266</v>
       </c>
       <c r="H22" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="23" ht="15">
@@ -1694,47 +1703,47 @@
         <v>9</v>
       </c>
       <c r="C23" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D23" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="24" ht="15">
       <c r="A24" s="5" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C24" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D24" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="25" ht="15">
       <c r="A25" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C25" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E25" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="26" ht="15">
@@ -1742,36 +1751,36 @@
         <v>27</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C26" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D26" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="27" ht="15">
       <c r="A27" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B27" t="s">
+        <v>105</v>
+      </c>
+      <c r="C27" t="s">
+        <v>106</v>
+      </c>
+      <c r="D27" t="s">
+        <v>107</v>
+      </c>
+      <c r="E27" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="C27" t="s">
-        <v>105</v>
-      </c>
-      <c r="D27" t="s">
-        <v>106</v>
-      </c>
-      <c r="E27" s="4" t="s">
-        <v>103</v>
-      </c>
       <c r="F27" s="7" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="G27" s="1">
         <v>46111</v>
@@ -1779,46 +1788,46 @@
     </row>
     <row r="28" ht="15">
       <c r="A28" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B28" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C28" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D28" t="s">
         <v>10</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H28" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="29" ht="15">
       <c r="A29" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B29" t="s">
         <v>9</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D29" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E29" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F29" s="10"/>
       <c r="G29" s="1">
         <v>46023</v>
       </c>
       <c r="H29" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="30" ht="15">
@@ -1826,19 +1835,19 @@
         <v>27</v>
       </c>
       <c r="B30" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C30" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D30" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E30" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="31" ht="15">
@@ -1849,16 +1858,16 @@
         <v>9</v>
       </c>
       <c r="C31" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D31" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E31" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G31" s="1">
         <v>46164</v>
@@ -1866,42 +1875,46 @@
     </row>
     <row r="32" ht="15">
       <c r="A32" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B32" t="s">
         <v>9</v>
       </c>
       <c r="C32" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D32" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E32" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F32" s="7" t="s">
-        <v>125</v>
-      </c>
+        <v>126</v>
+      </c>
+      <c r="G32" s="1"/>
     </row>
     <row r="33" ht="15">
       <c r="A33" s="5" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C33" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D33" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E33" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>129</v>
+        <v>130</v>
+      </c>
+      <c r="G33" s="1">
+        <v>46159</v>
       </c>
     </row>
     <row r="34" ht="15">
@@ -1912,16 +1925,16 @@
         <v>23</v>
       </c>
       <c r="C34" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D34" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E34" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F34" s="7" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="35" ht="15">
@@ -1932,13 +1945,13 @@
         <v>9</v>
       </c>
       <c r="C35" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D35" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E35" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="36" ht="15">
@@ -1954,24 +1967,25 @@
     <hyperlink r:id="rId2" ref="F3"/>
     <hyperlink r:id="rId3" ref="F4"/>
     <hyperlink r:id="rId4" ref="F5"/>
-    <hyperlink r:id="rId5" ref="F10" tooltip="https://www.unifr.ch/phys/en/department/jobs/"/>
-    <hyperlink r:id="rId6" ref="F11"/>
-    <hyperlink r:id="rId7" ref="F13"/>
-    <hyperlink r:id="rId8" ref="F14"/>
-    <hyperlink r:id="rId9" ref="F15"/>
-    <hyperlink r:id="rId10" ref="F16"/>
-    <hyperlink r:id="rId11" ref="F17"/>
-    <hyperlink r:id="rId12" ref="F27"/>
-    <hyperlink r:id="rId13" ref="F31"/>
-    <hyperlink r:id="rId14" ref="F32"/>
-    <hyperlink r:id="rId15" ref="F33"/>
-    <hyperlink r:id="rId16" ref="F34"/>
+    <hyperlink r:id="rId5" ref="F6"/>
+    <hyperlink r:id="rId6" ref="F10" tooltip="https://www.unifr.ch/phys/en/department/jobs/"/>
+    <hyperlink r:id="rId7" ref="F11"/>
+    <hyperlink r:id="rId8" ref="F13"/>
+    <hyperlink r:id="rId9" ref="F14"/>
+    <hyperlink r:id="rId10" ref="F15"/>
+    <hyperlink r:id="rId11" ref="F16"/>
+    <hyperlink r:id="rId12" ref="F17"/>
+    <hyperlink r:id="rId13" ref="F27"/>
+    <hyperlink r:id="rId14" ref="F31"/>
+    <hyperlink r:id="rId15" ref="F32"/>
+    <hyperlink r:id="rId16" ref="F33"/>
+    <hyperlink r:id="rId17" ref="F34"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="0" verticalDpi="0" copies="1"/>
   <headerFooter/>
-  <legacyDrawing r:id="rId19"/>
+  <legacyDrawing r:id="rId20"/>
 </worksheet>
 </file>
 
@@ -1984,37 +1998,37 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="11" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
   </sheetData>

</xml_diff>